<commit_message>
refactor and bad model
</commit_message>
<xml_diff>
--- a/rankings.xlsx
+++ b/rankings.xlsx
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="161">

</xml_diff>